<commit_message>
Wire cumNIRef + actual facility costs + correct debt service to all 5 dashboard call sites
Dashboard improvements:
- Break-even formula marks only the first year cumNI goes non-negative
- Revenue Sources shows per-year counts with conditional formatting
- Cash Runway shows per-year months with conditional formatting
- Facility % uses actual occupancy_facility category costs
- V1 underwriting dashboard now uses debt-service-only array (was capDebt total)

Shared benchmark-thresholds.ts module (single source of truth):
- Extracted BENCHMARK_* constants; financial-health.ts and workbook-helpers.ts
  both import from this shared module (no more magic numbers or duplication)

computeFacilityCostByYear uses Pick<ExpenseRow,...> for type-safe call sites.
buildFiveYearPL return type includes cumNIRow.
ModelData.currentYearProjection added to excel-export.ts interface.

Typecheck clean (0 errors), 24/24 excel QA, 33/33 parity.
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Underwriting_V1_(14-tab)_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Underwriting_V1_(14-tab)_Charter_ADA_Grade-Band.xlsx
@@ -990,7 +990,7 @@
     <t>Debt Affordability</t>
   </si>
   <si>
-    <t>DSCR of 55.03x provides comfortable coverage of debt payments with room to spare.</t>
+    <t>DSCR of 66.83x provides comfortable coverage of debt payments with room to spare.</t>
   </si>
   <si>
     <t>Maintain this ratio as you take on any additional debt.</t>
@@ -1008,7 +1008,7 @@
     <t>Reserve Strength</t>
   </si>
   <si>
-    <t>34.2 months of reserves by Year 5 — a strong buffer for unexpected costs.</t>
+    <t>34.3 months of reserves by Year 5 — a strong buffer for unexpected costs.</t>
   </si>
   <si>
     <t>Continue growing reserves toward 6 months for best-in-class financial health.</t>
@@ -3957,19 +3957,19 @@
         <v>164</v>
       </c>
       <c r="C11" s="61">
-        <v>106629</v>
+        <v>46629</v>
       </c>
       <c r="D11" s="61">
-        <v>66629</v>
+        <v>46629</v>
       </c>
       <c r="E11" s="61">
-        <v>71629</v>
+        <v>46629</v>
       </c>
       <c r="F11" s="61">
-        <v>56629</v>
+        <v>46629</v>
       </c>
       <c r="G11" s="61">
-        <v>56629</v>
+        <v>46629</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -4152,19 +4152,19 @@
         <v>194</v>
       </c>
       <c r="C20" s="71">
-        <v>-0.9897401269823406</v>
+        <v>-2.2632910849471357</v>
       </c>
       <c r="D20" s="72">
-        <v>7.521469630341143</v>
+        <v>10.74756053100002</v>
       </c>
       <c r="E20" s="72">
-        <v>18.630582585265746</v>
+        <v>28.619314160715433</v>
       </c>
       <c r="F20" s="72">
-        <v>38.49596496494729</v>
+        <v>46.751763923738444</v>
       </c>
       <c r="G20" s="72">
-        <v>55.0267354182486</v>
+        <v>66.82770378948723</v>
       </c>
       <c r="H20" s="69" t="s">
         <v>288</v>

</xml_diff>

<commit_message>
Improve financial model by detailing revenue streams per program
Update generated workbooks to display program-level revenue breakdowns and ensure formula integrity across all financial statements.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9c21ea3d-f26d-4d80-a097-4fdf87eda33a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/IGIVAYe
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Underwriting_V1_(14-tab)_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Underwriting_V1_(14-tab)_Charter_ADA_Grade-Band.xlsx
@@ -990,7 +990,7 @@
     <t>Debt Affordability</t>
   </si>
   <si>
-    <t>DSCR of 55.03x provides comfortable coverage of debt payments with room to spare.</t>
+    <t>DSCR of 66.83x provides comfortable coverage of debt payments with room to spare.</t>
   </si>
   <si>
     <t>Maintain this ratio as you take on any additional debt.</t>
@@ -1008,7 +1008,7 @@
     <t>Reserve Strength</t>
   </si>
   <si>
-    <t>34.2 months of reserves by Year 5 — a strong buffer for unexpected costs.</t>
+    <t>34.3 months of reserves by Year 5 — a strong buffer for unexpected costs.</t>
   </si>
   <si>
     <t>Continue growing reserves toward 6 months for best-in-class financial health.</t>
@@ -3957,19 +3957,19 @@
         <v>164</v>
       </c>
       <c r="C11" s="61">
-        <v>106629</v>
+        <v>46629</v>
       </c>
       <c r="D11" s="61">
-        <v>66629</v>
+        <v>46629</v>
       </c>
       <c r="E11" s="61">
-        <v>71629</v>
+        <v>46629</v>
       </c>
       <c r="F11" s="61">
-        <v>56629</v>
+        <v>46629</v>
       </c>
       <c r="G11" s="61">
-        <v>56629</v>
+        <v>46629</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -4152,19 +4152,19 @@
         <v>194</v>
       </c>
       <c r="C20" s="71">
-        <v>-0.9897401269823406</v>
+        <v>-2.2632910849471357</v>
       </c>
       <c r="D20" s="72">
-        <v>7.521469630341143</v>
+        <v>10.74756053100002</v>
       </c>
       <c r="E20" s="72">
-        <v>18.630582585265746</v>
+        <v>28.619314160715433</v>
       </c>
       <c r="F20" s="72">
-        <v>38.49596496494729</v>
+        <v>46.751763923738444</v>
       </c>
       <c r="G20" s="72">
-        <v>55.0267354182486</v>
+        <v>66.82770378948723</v>
       </c>
       <c r="H20" s="69" t="s">
         <v>288</v>

</xml_diff>